<commit_message>
added a bunch of features bro, pull it and find out lol
</commit_message>
<xml_diff>
--- a/finance_tracker.xlsx
+++ b/finance_tracker.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,6 +495,11 @@
           <t>Amount</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -513,6 +518,7 @@
       <c r="D2" t="n">
         <v>1268</v>
       </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -530,6 +536,87 @@
       </c>
       <c r="D3" t="n">
         <v>1290</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>878</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2794</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Clothing</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2249</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>90</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Badminton court booking</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -543,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,6 +681,27 @@
         <v>10000</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GOLDBEES NSE</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>113</v>
+      </c>
+      <c r="E3" t="n">
+        <v>15000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added a bunch of new features including income, updated stats in dahsboards and a better prompt to generate a full report
</commit_message>
<xml_diff>
--- a/finance_tracker.xlsx
+++ b/finance_tracker.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="MAIN SALARY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="EXPENSES" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="SHARES and FUNDS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="OTHER INCOME" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EXPENSES" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SHARES and FUNDS" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -471,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,7 +488,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Expense Type</t>
+          <t>Income Type</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -507,18 +508,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Food</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1268</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>360</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Refund for the tee that I ordered with badminton shoes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -526,96 +531,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Settlements</t>
+          <t>Gift</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1290</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-03-04</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Gift</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>878</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Gift</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>2794</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>2249</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Sports</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>90</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Badminton court booking</t>
+        <v>3000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Grandparents gave some mone</t>
         </is>
       </c>
     </row>
@@ -630,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -646,17 +575,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Share/Fund Name</t>
+          <t>Expense Type</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Total Amount Invested</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -666,20 +595,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GOLDBEESNSE</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>72</v>
-      </c>
-      <c r="E2" t="n">
-        <v>10000</v>
-      </c>
+        <v>1268</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -687,12 +614,231 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1290</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>878</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Gift for grandparenst</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2794</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Gift for parents</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Clothing</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2249</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Badminton shoes, tshirts, shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>2026-03-10</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>90</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Badminton court booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>900</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Go Karting</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>250</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Petrol</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sr No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share/Fund Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Total Amount Invested</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GOLDBEESNSE</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>72</v>
+      </c>
+      <c r="E2" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GOLDBEES NSE</t>
+          <t>GOLDBEESNSE</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -700,6 +846,27 @@
       </c>
       <c r="E3" t="n">
         <v>15000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TATAINVEST.NS</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added budgets, recurring expenses, import and changed the entire UI for better data handling
</commit_message>
<xml_diff>
--- a/finance_tracker.xlsx
+++ b/finance_tracker.xlsx
@@ -776,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -805,6 +805,11 @@
           <t>Total Amount Invested</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -817,7 +822,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GOLDBEESNSE</t>
+          <t>GOLDBEES</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -825,6 +830,11 @@
       </c>
       <c r="E2" t="n">
         <v>10000</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>GOLDBEES.NS</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -838,7 +848,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GOLDBEESNSE</t>
+          <t>GOLDBEES</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -846,6 +856,11 @@
       </c>
       <c r="E3" t="n">
         <v>15000</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>GOLDBEES.NS</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -859,7 +874,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TATAINVEST.NS</t>
+          <t>TATAINV</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -867,6 +882,11 @@
       </c>
       <c r="E4" t="n">
         <v>3000</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>TATAINVEST.NS</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>